<commit_message>
Results: updating experimental results
</commit_message>
<xml_diff>
--- a/src/evaluation/data/Backup/qwen25_7b_validation/comparison.xlsx
+++ b/src/evaluation/data/Backup/qwen25_7b_validation/comparison.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Uni-Köln\Masterarbeit\Software\uzk-masterarbeit\src\evaluation\data\Backup\qwen25_7b_validation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D10502E4-F08C-4349-9A33-D8A38AA6DD05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9E46671-EEF3-47B4-9376-B757284CD320}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,10 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="156">
-  <si>
-    <t>gpt-4.a-mini</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="492" uniqueCount="156">
   <si>
     <t>run1</t>
   </si>
@@ -634,6 +631,9 @@
   </si>
   <si>
     <t>p-Value</t>
+  </si>
+  <si>
+    <t>gpt-4.1-mini</t>
   </si>
 </sst>
 </file>
@@ -1677,35 +1677,35 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>155</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
         <v>2</v>
       </c>
-      <c r="D3" t="s">
+      <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="F3" t="s">
-        <v>4</v>
-      </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I3" t="s">
         <v>15</v>
       </c>
-      <c r="H3" t="s">
-        <v>16</v>
-      </c>
-      <c r="I3" t="s">
-        <v>155</v>
+      <c r="J3" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B4">
         <v>0.66156887149880883</v>
@@ -1720,21 +1720,24 @@
         <f>AVERAGE(B4:D4)</f>
         <v>0.66485917558904195</v>
       </c>
-      <c r="G4">
+      <c r="G4" t="s">
+        <v>4</v>
+      </c>
+      <c r="H4">
         <v>0.53558362800000003</v>
       </c>
-      <c r="H4">
+      <c r="I4">
         <f>PEARSON('[1]Human Details'!$J$2:$J$16, '[1]gpt-4.1-mini-Details'!$J$2:$J$16)</f>
         <v>0.73322697783828605</v>
       </c>
-      <c r="I4">
+      <c r="J4">
         <f>_xlfn.T.TEST('Human Details'!J2:J16, 'gpt-4.1-mini Details'!J2:J16,2,1)</f>
         <v>7.955926097945934E-2</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B5">
         <v>0.62444581280788181</v>
@@ -1749,21 +1752,24 @@
         <f t="shared" ref="F5:F12" si="0">AVERAGE(B5:D5)</f>
         <v>0.63196496989600448</v>
       </c>
-      <c r="G5">
+      <c r="G5" t="s">
+        <v>5</v>
+      </c>
+      <c r="H5">
         <v>0.58594568300000005</v>
       </c>
-      <c r="H5">
+      <c r="I5">
         <f>PEARSON('[1]Human Details'!$K$2:$K$16, '[1]gpt-4.1-mini-Details'!$K$2:$K$16)</f>
         <v>0.56215486685579941</v>
       </c>
-      <c r="I5">
+      <c r="J5">
         <f>_xlfn.T.TEST('Human Details'!K2:K16, 'gpt-4.1-mini Details'!K2:K16,2,1)</f>
         <v>0.28661464799529518</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B6">
         <v>0.62411398464630641</v>
@@ -1778,21 +1784,24 @@
         <f t="shared" si="0"/>
         <v>0.61850217249724604</v>
       </c>
-      <c r="G6">
+      <c r="G6" t="s">
+        <v>6</v>
+      </c>
+      <c r="H6">
         <v>0.503276689</v>
       </c>
-      <c r="H6">
+      <c r="I6">
         <f>PEARSON('[1]Human Details'!$L$2:$L$16, '[1]gpt-4.1-mini-Details'!$L$2:$L$16)</f>
         <v>0.55107579992168187</v>
       </c>
-      <c r="I6">
+      <c r="J6">
         <f>_xlfn.T.TEST('Human Details'!L2:L16, 'gpt-4.1-mini Details'!L2:L16,2,1)</f>
         <v>8.4748450378080487E-2</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B7">
         <v>0.75828297912577958</v>
@@ -1807,21 +1816,24 @@
         <f t="shared" si="0"/>
         <v>0.7588076597258181</v>
       </c>
-      <c r="G7">
+      <c r="G7" t="s">
+        <v>7</v>
+      </c>
+      <c r="H7">
         <v>0.24528230000000001</v>
       </c>
-      <c r="H7">
+      <c r="I7">
         <f>PEARSON('[1]Human Details'!$M$2:$M$16, '[1]gpt-4.1-mini-Details'!$M$2:$M$16)</f>
         <v>0.26938296177516874</v>
       </c>
-      <c r="I7">
+      <c r="J7">
         <f>_xlfn.T.TEST('Human Details'!M2:M16, 'gpt-4.1-mini Details'!M2:M16,2,1)</f>
         <v>3.3677965720193662E-5</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B8">
         <v>0.27292447328324371</v>
@@ -1836,21 +1848,24 @@
         <f t="shared" si="0"/>
         <v>0.26950926621229687</v>
       </c>
-      <c r="G8">
+      <c r="G8" t="s">
+        <v>8</v>
+      </c>
+      <c r="H8">
         <v>0.40351567199999999</v>
       </c>
-      <c r="H8">
+      <c r="I8">
         <f>PEARSON('[1]Human Details'!$N$2:$N$16, '[1]gpt-4.1-mini-Details'!$N$2:$N$16)</f>
         <v>0.36082995651787875</v>
       </c>
-      <c r="I8">
+      <c r="J8">
         <f>_xlfn.T.TEST('Human Details'!N2:N16, 'gpt-4.1-mini Details'!N2:N16,2,1)</f>
         <v>0.6988549756964495</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B9">
         <v>0.59892572244511921</v>
@@ -1865,21 +1880,24 @@
         <f t="shared" si="0"/>
         <v>0.59861098158178683</v>
       </c>
-      <c r="G9">
+      <c r="G9" t="s">
+        <v>9</v>
+      </c>
+      <c r="H9">
         <v>0.44812488099999997</v>
       </c>
-      <c r="H9">
+      <c r="I9">
         <f>PEARSON('[1]Human Details'!$O$2:$O$16, '[1]gpt-4.1-mini-Details'!$O$2:$O$16)</f>
         <v>0.46513087562715405</v>
       </c>
-      <c r="I9">
+      <c r="J9">
         <f>_xlfn.T.TEST('Human Details'!O2:O16, 'gpt-4.1-mini Details'!O2:O16,2,1)</f>
         <v>0.17697202988021674</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B10">
         <v>0.3466954022988506</v>
@@ -1897,7 +1915,7 @@
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B11">
         <v>0.50862068965517238</v>
@@ -1915,7 +1933,7 @@
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B12">
         <v>12.829803801816089</v>
@@ -1959,35 +1977,35 @@
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C17" t="s">
+        <v>1</v>
+      </c>
+      <c r="D17" t="s">
         <v>2</v>
       </c>
-      <c r="D17" t="s">
+      <c r="F17" t="s">
         <v>3</v>
       </c>
-      <c r="F17" t="s">
-        <v>4</v>
-      </c>
       <c r="G17" t="s">
+        <v>14</v>
+      </c>
+      <c r="H17" t="s">
         <v>15</v>
       </c>
-      <c r="H17" t="s">
-        <v>16</v>
-      </c>
       <c r="I17" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B18">
         <v>0.64263006338899198</v>
@@ -2017,7 +2035,7 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B19">
         <v>0.68697722567287778</v>
@@ -2047,7 +2065,7 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B20">
         <v>0.71522946857201253</v>
@@ -2077,7 +2095,7 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B21">
         <v>0.76445786427386186</v>
@@ -2107,7 +2125,7 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B22">
         <v>0.112832086749091</v>
@@ -2136,7 +2154,7 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B23">
         <v>0.53499107956067182</v>
@@ -2166,7 +2184,7 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B24">
         <v>0.31057971014492758</v>
@@ -2184,7 +2202,7 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B25">
         <v>0.46086956521739131</v>
@@ -2202,7 +2220,7 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B26">
         <v>11.52793571223383</v>
@@ -2249,82 +2267,82 @@
   <sheetData>
     <row r="1" spans="1:26" ht="90" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="P1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="J1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="O1" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="P1" s="2" t="s">
+      <c r="Q1" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="R1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="R1" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="S1" s="2" t="s">
+      <c r="T1" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="U1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="V1" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="V1" s="2" t="s">
+      <c r="W1" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="W1" s="2" t="s">
+      <c r="X1" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="X1" s="2" t="s">
+      <c r="Y1" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="Y1" s="2" t="s">
+      <c r="Z1" s="2" t="s">
         <v>34</v>
-      </c>
-      <c r="Z1" s="2" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="2" spans="1:26" ht="409.5" x14ac:dyDescent="0.25">
@@ -2332,28 +2350,28 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2" t="s">
         <v>36</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="F2" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="H2" t="s">
         <v>41</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>42</v>
-      </c>
-      <c r="I2" t="s">
-        <v>43</v>
       </c>
       <c r="J2" s="1">
         <v>1</v>
@@ -2390,13 +2408,13 @@
         <v>45.547114849090583</v>
       </c>
       <c r="U2" t="s">
+        <v>43</v>
+      </c>
+      <c r="V2" t="s">
         <v>44</v>
       </c>
-      <c r="V2" t="s">
+      <c r="W2" t="s">
         <v>45</v>
-      </c>
-      <c r="W2" t="s">
-        <v>46</v>
       </c>
       <c r="X2">
         <v>5</v>
@@ -2405,7 +2423,7 @@
         <v>6</v>
       </c>
       <c r="Z2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:26" ht="409.5" x14ac:dyDescent="0.25">
@@ -2413,28 +2431,28 @@
         <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="F3" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="G3" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="H3" t="s">
         <v>52</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>53</v>
-      </c>
-      <c r="I3" t="s">
-        <v>54</v>
       </c>
       <c r="J3" s="1">
         <v>0.5</v>
@@ -2471,7 +2489,7 @@
         <v>10.010499954223629</v>
       </c>
       <c r="Z3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="409.5" x14ac:dyDescent="0.25">
@@ -2479,28 +2497,28 @@
         <v>11</v>
       </c>
       <c r="B4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="C4" t="s">
-        <v>37</v>
-      </c>
-      <c r="D4" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="F4" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="G4" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="H4" t="s">
         <v>60</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>61</v>
-      </c>
-      <c r="I4" t="s">
-        <v>62</v>
       </c>
       <c r="J4" s="1">
         <f>0.5</f>
@@ -2538,10 +2556,10 @@
         <v>9.4738509654998779</v>
       </c>
       <c r="U4" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="V4" s="4" t="s">
         <v>63</v>
-      </c>
-      <c r="V4" s="4" t="s">
-        <v>64</v>
       </c>
       <c r="X4">
         <v>3</v>
@@ -2555,28 +2573,28 @@
         <v>17</v>
       </c>
       <c r="B5" t="s">
+        <v>64</v>
+      </c>
+      <c r="C5" t="s">
         <v>65</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="E5" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="F5" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="G5" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="H5" t="s">
         <v>70</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>71</v>
-      </c>
-      <c r="I5" t="s">
-        <v>72</v>
       </c>
       <c r="J5" s="1">
         <f>2/3</f>
@@ -2615,13 +2633,13 @@
         <v>7.7230634689331046</v>
       </c>
       <c r="U5" t="s">
+        <v>72</v>
+      </c>
+      <c r="V5" t="s">
         <v>73</v>
       </c>
-      <c r="V5" t="s">
+      <c r="W5" t="s">
         <v>74</v>
-      </c>
-      <c r="W5" t="s">
-        <v>75</v>
       </c>
       <c r="X5">
         <v>3</v>
@@ -2630,7 +2648,7 @@
         <v>6</v>
       </c>
       <c r="Z5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6" spans="1:26" ht="409.5" x14ac:dyDescent="0.25">
@@ -2638,28 +2656,28 @@
         <v>20</v>
       </c>
       <c r="B6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D6" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="E6" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="F6" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="G6" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="G6" s="3" t="s">
+      <c r="H6" t="s">
         <v>80</v>
       </c>
-      <c r="H6" t="s">
-        <v>81</v>
-      </c>
       <c r="I6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J6" s="1">
         <v>0.9</v>
@@ -2695,7 +2713,7 @@
         <v>8.7654869556427002</v>
       </c>
       <c r="Z6" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="7" spans="1:26" ht="409.5" x14ac:dyDescent="0.25">
@@ -2703,28 +2721,28 @@
         <v>30</v>
       </c>
       <c r="B7" t="s">
+        <v>82</v>
+      </c>
+      <c r="C7" t="s">
+        <v>65</v>
+      </c>
+      <c r="D7" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="C7" t="s">
-        <v>66</v>
-      </c>
-      <c r="D7" s="3" t="s">
+      <c r="E7" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="F7" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="G7" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="G7" s="3" t="s">
+      <c r="H7" t="s">
         <v>87</v>
       </c>
-      <c r="H7" t="s">
+      <c r="I7" t="s">
         <v>88</v>
-      </c>
-      <c r="I7" t="s">
-        <v>89</v>
       </c>
       <c r="J7" s="1">
         <f>2/6</f>
@@ -2762,7 +2780,7 @@
         <v>9.9265642166137695</v>
       </c>
       <c r="Z7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="409.5" x14ac:dyDescent="0.25">
@@ -2770,28 +2788,28 @@
         <v>33</v>
       </c>
       <c r="B8" t="s">
+        <v>90</v>
+      </c>
+      <c r="C8" t="s">
+        <v>65</v>
+      </c>
+      <c r="D8" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="C8" t="s">
-        <v>66</v>
-      </c>
-      <c r="D8" s="3" t="s">
+      <c r="E8" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="F8" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="G8" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="G8" s="3" t="s">
+      <c r="H8" t="s">
         <v>95</v>
       </c>
-      <c r="H8" t="s">
-        <v>96</v>
-      </c>
       <c r="I8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J8" s="1">
         <v>0.5</v>
@@ -2832,28 +2850,28 @@
         <v>34</v>
       </c>
       <c r="B9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D9" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="E9" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="F9" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="G9" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="G9" s="3" t="s">
+      <c r="H9" t="s">
         <v>100</v>
       </c>
-      <c r="H9" t="s">
-        <v>101</v>
-      </c>
       <c r="I9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="J9" s="1">
         <v>0</v>
@@ -2894,28 +2912,28 @@
         <v>64</v>
       </c>
       <c r="B10" t="s">
+        <v>101</v>
+      </c>
+      <c r="C10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D10" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="C10" t="s">
-        <v>37</v>
-      </c>
-      <c r="D10" s="3" t="s">
+      <c r="E10" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="F10" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="G10" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="G10" s="3" t="s">
+      <c r="H10" t="s">
         <v>106</v>
       </c>
-      <c r="H10" t="s">
-        <v>107</v>
-      </c>
       <c r="I10" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="J10" s="1">
         <v>0</v>
@@ -2957,28 +2975,28 @@
         <v>65</v>
       </c>
       <c r="B11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C11" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D11" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="E11" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="F11" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="F11" s="3" t="s">
+      <c r="G11" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="G11" s="3" t="s">
+      <c r="H11" t="s">
         <v>111</v>
       </c>
-      <c r="H11" t="s">
+      <c r="I11" t="s">
         <v>112</v>
-      </c>
-      <c r="I11" t="s">
-        <v>113</v>
       </c>
       <c r="J11" s="1">
         <f>4/6</f>
@@ -3020,28 +3038,28 @@
         <v>84</v>
       </c>
       <c r="B12" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D12" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="E12" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="F12" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="F12" s="3" t="s">
+      <c r="G12" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="G12" s="3" t="s">
+      <c r="H12" t="s">
         <v>117</v>
       </c>
-      <c r="H12" t="s">
-        <v>118</v>
-      </c>
       <c r="I12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J12" s="1">
         <f>5/7</f>
@@ -3086,7 +3104,7 @@
         <v>31</v>
       </c>
       <c r="Z12" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="409.5" x14ac:dyDescent="0.25">
@@ -3094,28 +3112,28 @@
         <v>89</v>
       </c>
       <c r="B13" t="s">
+        <v>119</v>
+      </c>
+      <c r="C13" t="s">
+        <v>65</v>
+      </c>
+      <c r="D13" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="C13" t="s">
-        <v>66</v>
-      </c>
-      <c r="D13" s="3" t="s">
+      <c r="E13" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="E13" s="3" t="s">
+      <c r="F13" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="F13" s="3" t="s">
+      <c r="G13" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="G13" s="3" t="s">
+      <c r="H13" t="s">
         <v>124</v>
       </c>
-      <c r="H13" t="s">
+      <c r="I13" t="s">
         <v>125</v>
-      </c>
-      <c r="I13" t="s">
-        <v>126</v>
       </c>
       <c r="J13" s="1">
         <v>0</v>
@@ -3152,7 +3170,7 @@
         <v>8.4058101177215576</v>
       </c>
       <c r="Z13" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="14" spans="1:26" ht="409.5" x14ac:dyDescent="0.25">
@@ -3160,28 +3178,28 @@
         <v>91</v>
       </c>
       <c r="B14" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C14" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D14" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="E14" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="E14" s="3" t="s">
+      <c r="F14" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="F14" s="3" t="s">
+      <c r="G14" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="G14" s="3" t="s">
+      <c r="H14" t="s">
         <v>131</v>
       </c>
-      <c r="H14" t="s">
-        <v>132</v>
-      </c>
       <c r="I14" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="J14" s="1">
         <f>6/13</f>
@@ -3221,13 +3239,13 @@
         <v>14.452758550643919</v>
       </c>
       <c r="U14" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="V14" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="V14" s="5" t="s">
+      <c r="W14" s="5" t="s">
         <v>134</v>
-      </c>
-      <c r="W14" s="5" t="s">
-        <v>135</v>
       </c>
       <c r="X14">
         <v>17</v>
@@ -3236,7 +3254,7 @@
         <v>9</v>
       </c>
       <c r="Z14" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="409.5" x14ac:dyDescent="0.25">
@@ -3244,28 +3262,28 @@
         <v>97</v>
       </c>
       <c r="B15" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C15" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D15" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E15" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="E15" s="3" t="s">
+      <c r="F15" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="F15" s="3" t="s">
+      <c r="G15" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="G15" s="3" t="s">
+      <c r="H15" t="s">
         <v>140</v>
       </c>
-      <c r="H15" t="s">
-        <v>141</v>
-      </c>
       <c r="I15" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="J15" s="1">
         <f>4/10</f>
@@ -3305,13 +3323,13 @@
         <v>15.475528955459589</v>
       </c>
       <c r="U15" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="V15" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="V15" s="5" t="s">
+      <c r="W15" s="5" t="s">
         <v>143</v>
-      </c>
-      <c r="W15" s="5" t="s">
-        <v>144</v>
       </c>
       <c r="X15">
         <v>12</v>
@@ -3320,7 +3338,7 @@
         <v>8</v>
       </c>
       <c r="Z15" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="16" spans="1:26" ht="409.5" x14ac:dyDescent="0.25">
@@ -3328,28 +3346,28 @@
         <v>110</v>
       </c>
       <c r="B16" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C16" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D16" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="E16" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="F16" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="F16" s="3" t="s">
+      <c r="G16" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="G16" s="3" t="s">
+      <c r="H16" t="s">
         <v>149</v>
       </c>
-      <c r="H16" t="s">
+      <c r="I16" t="s">
         <v>150</v>
-      </c>
-      <c r="I16" t="s">
-        <v>151</v>
       </c>
       <c r="J16" s="1">
         <f>3/12</f>
@@ -3389,13 +3407,13 @@
         <v>16.019131183624271</v>
       </c>
       <c r="U16" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="V16" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="V16" s="5" t="s">
+      <c r="W16" s="5" t="s">
         <v>153</v>
-      </c>
-      <c r="W16" s="5" t="s">
-        <v>154</v>
       </c>
       <c r="X16">
         <v>5</v>
@@ -3426,64 +3444,64 @@
   <sheetData>
     <row r="1" spans="1:20" ht="45" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="P1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="J1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="O1" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="P1" s="2" t="s">
+      <c r="Q1" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="R1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="R1" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="S1" s="2" t="s">
+      <c r="T1" s="2" t="s">
         <v>28</v>
-      </c>
-      <c r="T1" s="2" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:20" ht="409.5" x14ac:dyDescent="0.25">
@@ -3491,28 +3509,28 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2" t="s">
         <v>36</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="F2" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="H2" t="s">
         <v>41</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>42</v>
-      </c>
-      <c r="I2" t="s">
-        <v>43</v>
       </c>
       <c r="J2" s="8">
         <v>0.94444444444444442</v>
@@ -3553,28 +3571,28 @@
         <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="F3" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="G3" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="H3" t="s">
         <v>52</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>53</v>
-      </c>
-      <c r="I3" t="s">
-        <v>54</v>
       </c>
       <c r="J3" s="9">
         <v>0.5</v>
@@ -3615,28 +3633,28 @@
         <v>11</v>
       </c>
       <c r="B4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="C4" t="s">
-        <v>37</v>
-      </c>
-      <c r="D4" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="F4" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="G4" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="H4" t="s">
         <v>60</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>61</v>
-      </c>
-      <c r="I4" t="s">
-        <v>62</v>
       </c>
       <c r="J4" s="8">
         <v>0.83333333333333337</v>
@@ -3677,28 +3695,28 @@
         <v>17</v>
       </c>
       <c r="B5" t="s">
+        <v>64</v>
+      </c>
+      <c r="C5" t="s">
         <v>65</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="E5" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="F5" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="G5" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="H5" t="s">
         <v>70</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>71</v>
-      </c>
-      <c r="I5" t="s">
-        <v>72</v>
       </c>
       <c r="J5" s="8">
         <v>0.8</v>
@@ -3739,28 +3757,28 @@
         <v>20</v>
       </c>
       <c r="B6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D6" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="E6" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="F6" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="G6" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="G6" s="3" t="s">
+      <c r="H6" t="s">
         <v>80</v>
       </c>
-      <c r="H6" t="s">
-        <v>81</v>
-      </c>
       <c r="I6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J6" s="10">
         <v>0.6</v>
@@ -3801,28 +3819,28 @@
         <v>30</v>
       </c>
       <c r="B7" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C7" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D7" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="E7" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="F7" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="G7" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="G7" s="3" t="s">
+      <c r="H7" t="s">
         <v>95</v>
       </c>
-      <c r="H7" t="s">
-        <v>96</v>
-      </c>
       <c r="I7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J7" s="8">
         <v>1</v>
@@ -3863,28 +3881,28 @@
         <v>33</v>
       </c>
       <c r="B8" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C8" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D8" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="E8" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="F8" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="G8" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="G8" s="3" t="s">
+      <c r="H8" t="s">
         <v>100</v>
       </c>
-      <c r="H8" t="s">
-        <v>101</v>
-      </c>
       <c r="I8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="J8" s="8">
         <v>0.83333333333333337</v>
@@ -3925,28 +3943,28 @@
         <v>34</v>
       </c>
       <c r="B9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D9" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="E9" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="F9" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="G9" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="G9" s="3" t="s">
+      <c r="H9" t="s">
         <v>106</v>
       </c>
-      <c r="H9" t="s">
-        <v>107</v>
-      </c>
       <c r="I9" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="J9" s="9">
         <v>0</v>
@@ -3987,28 +4005,28 @@
         <v>64</v>
       </c>
       <c r="B10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C10" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D10" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="E10" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="F10" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="G10" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="G10" s="3" t="s">
+      <c r="H10" t="s">
         <v>111</v>
       </c>
-      <c r="H10" t="s">
+      <c r="I10" t="s">
         <v>112</v>
-      </c>
-      <c r="I10" t="s">
-        <v>113</v>
       </c>
       <c r="J10" s="9">
         <v>0</v>
@@ -4049,28 +4067,28 @@
         <v>65</v>
       </c>
       <c r="B11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C11" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D11" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="E11" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="F11" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="F11" s="3" t="s">
+      <c r="G11" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="G11" s="3" t="s">
+      <c r="H11" t="s">
         <v>117</v>
       </c>
-      <c r="H11" t="s">
-        <v>118</v>
-      </c>
       <c r="I11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J11" s="9">
         <v>0.55555555555555558</v>
@@ -4111,28 +4129,28 @@
         <v>84</v>
       </c>
       <c r="B12" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D12" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="E12" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="F12" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="F12" s="3" t="s">
+      <c r="G12" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="G12" s="3" t="s">
+      <c r="H12" t="s">
         <v>124</v>
       </c>
-      <c r="H12" t="s">
+      <c r="I12" t="s">
         <v>125</v>
-      </c>
-      <c r="I12" t="s">
-        <v>126</v>
       </c>
       <c r="J12" s="8">
         <v>0.9285714285714286</v>
@@ -4173,28 +4191,28 @@
         <v>89</v>
       </c>
       <c r="B13" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C13" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D13" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="E13" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="E13" s="3" t="s">
+      <c r="F13" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="F13" s="3" t="s">
+      <c r="G13" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="G13" s="3" t="s">
+      <c r="H13" t="s">
         <v>131</v>
       </c>
-      <c r="H13" t="s">
-        <v>132</v>
-      </c>
       <c r="I13" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="J13" s="9">
         <v>0</v>
@@ -4235,28 +4253,28 @@
         <v>91</v>
       </c>
       <c r="B14" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C14" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D14" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E14" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="E14" s="3" t="s">
+      <c r="F14" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="F14" s="3" t="s">
+      <c r="G14" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="G14" s="3" t="s">
+      <c r="H14" t="s">
         <v>140</v>
       </c>
-      <c r="H14" t="s">
-        <v>141</v>
-      </c>
       <c r="I14" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="J14" s="9">
         <v>0.53846153846153844</v>
@@ -4297,28 +4315,28 @@
         <v>97</v>
       </c>
       <c r="B15" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C15" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D15" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="E15" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="E15" s="3" t="s">
+      <c r="F15" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="F15" s="3" t="s">
+      <c r="G15" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="G15" s="3" t="s">
+      <c r="H15" t="s">
         <v>149</v>
       </c>
-      <c r="H15" t="s">
+      <c r="I15" t="s">
         <v>150</v>
-      </c>
-      <c r="I15" t="s">
-        <v>151</v>
       </c>
       <c r="J15" s="8">
         <v>0.89473684210526316</v>
@@ -4359,28 +4377,28 @@
         <v>110</v>
       </c>
       <c r="B16" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C16" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D16" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="E16" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="F16" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="F16" s="3" t="s">
+      <c r="G16" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="G16" s="3" t="s">
+      <c r="H16" t="s">
         <v>87</v>
       </c>
-      <c r="H16" t="s">
+      <c r="I16" t="s">
         <v>88</v>
-      </c>
-      <c r="I16" t="s">
-        <v>89</v>
       </c>
       <c r="J16" s="9">
         <v>0.2857142857142857</v>
@@ -4447,64 +4465,64 @@
   <sheetData>
     <row r="1" spans="1:20" ht="45" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="P1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="J1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="O1" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="P1" s="2" t="s">
+      <c r="Q1" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="R1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="R1" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="S1" s="2" t="s">
+      <c r="T1" s="2" t="s">
         <v>28</v>
-      </c>
-      <c r="T1" s="2" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:20" ht="409.5" x14ac:dyDescent="0.25">
@@ -4512,28 +4530,28 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2" t="s">
         <v>36</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="F2" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="H2" t="s">
         <v>41</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>42</v>
-      </c>
-      <c r="I2" t="s">
-        <v>43</v>
       </c>
       <c r="J2" s="8">
         <v>0.8571428571428571</v>
@@ -4574,28 +4592,28 @@
         <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="F3" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="G3" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="H3" t="s">
         <v>52</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>53</v>
-      </c>
-      <c r="I3" t="s">
-        <v>54</v>
       </c>
       <c r="J3" s="9">
         <v>0.4</v>
@@ -4636,28 +4654,28 @@
         <v>11</v>
       </c>
       <c r="B4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="C4" t="s">
-        <v>37</v>
-      </c>
-      <c r="D4" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="F4" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="G4" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="H4" t="s">
         <v>60</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>61</v>
-      </c>
-      <c r="I4" t="s">
-        <v>62</v>
       </c>
       <c r="J4" s="9">
         <v>0.5</v>
@@ -4698,28 +4716,28 @@
         <v>17</v>
       </c>
       <c r="B5" t="s">
+        <v>64</v>
+      </c>
+      <c r="C5" t="s">
         <v>65</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="E5" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="F5" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="G5" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="H5" t="s">
         <v>70</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>71</v>
-      </c>
-      <c r="I5" t="s">
-        <v>72</v>
       </c>
       <c r="J5" s="9">
         <v>0.5</v>
@@ -4760,28 +4778,28 @@
         <v>20</v>
       </c>
       <c r="B6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D6" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="E6" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="F6" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="G6" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="G6" s="3" t="s">
+      <c r="H6" t="s">
         <v>80</v>
       </c>
-      <c r="H6" t="s">
-        <v>81</v>
-      </c>
       <c r="I6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J6" s="8">
         <v>0.8</v>
@@ -4822,28 +4840,28 @@
         <v>30</v>
       </c>
       <c r="B7" t="s">
+        <v>82</v>
+      </c>
+      <c r="C7" t="s">
+        <v>65</v>
+      </c>
+      <c r="D7" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="C7" t="s">
-        <v>66</v>
-      </c>
-      <c r="D7" s="3" t="s">
+      <c r="E7" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="F7" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="G7" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="G7" s="3" t="s">
+      <c r="H7" t="s">
         <v>87</v>
       </c>
-      <c r="H7" t="s">
+      <c r="I7" t="s">
         <v>88</v>
-      </c>
-      <c r="I7" t="s">
-        <v>89</v>
       </c>
       <c r="J7" s="9">
         <v>0.25</v>
@@ -4884,28 +4902,28 @@
         <v>33</v>
       </c>
       <c r="B8" t="s">
+        <v>90</v>
+      </c>
+      <c r="C8" t="s">
+        <v>65</v>
+      </c>
+      <c r="D8" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="C8" t="s">
-        <v>66</v>
-      </c>
-      <c r="D8" s="3" t="s">
+      <c r="E8" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="F8" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="G8" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="G8" s="3" t="s">
+      <c r="H8" t="s">
         <v>95</v>
       </c>
-      <c r="H8" t="s">
-        <v>96</v>
-      </c>
       <c r="I8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J8" s="9">
         <v>0.33333333333333331</v>
@@ -4946,28 +4964,28 @@
         <v>34</v>
       </c>
       <c r="B9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D9" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="E9" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="F9" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="G9" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="G9" s="3" t="s">
+      <c r="H9" t="s">
         <v>100</v>
       </c>
-      <c r="H9" t="s">
-        <v>101</v>
-      </c>
       <c r="I9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="J9" s="9">
         <v>0</v>
@@ -5008,28 +5026,28 @@
         <v>64</v>
       </c>
       <c r="B10" t="s">
+        <v>101</v>
+      </c>
+      <c r="C10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D10" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="C10" t="s">
-        <v>37</v>
-      </c>
-      <c r="D10" s="3" t="s">
+      <c r="E10" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="F10" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="G10" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="G10" s="3" t="s">
+      <c r="H10" t="s">
         <v>106</v>
       </c>
-      <c r="H10" t="s">
-        <v>107</v>
-      </c>
       <c r="I10" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="J10" s="8">
         <v>0.8</v>
@@ -5070,28 +5088,28 @@
         <v>65</v>
       </c>
       <c r="B11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C11" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D11" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="E11" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="F11" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="F11" s="3" t="s">
+      <c r="G11" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="G11" s="3" t="s">
+      <c r="H11" t="s">
         <v>111</v>
       </c>
-      <c r="H11" t="s">
+      <c r="I11" t="s">
         <v>112</v>
-      </c>
-      <c r="I11" t="s">
-        <v>113</v>
       </c>
       <c r="J11" s="10">
         <v>0.66666666666666663</v>
@@ -5132,28 +5150,28 @@
         <v>84</v>
       </c>
       <c r="B12" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D12" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="E12" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="F12" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="F12" s="3" t="s">
+      <c r="G12" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="G12" s="3" t="s">
+      <c r="H12" t="s">
         <v>117</v>
       </c>
-      <c r="H12" t="s">
-        <v>118</v>
-      </c>
       <c r="I12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J12" s="8">
         <v>0.8</v>
@@ -5194,28 +5212,28 @@
         <v>89</v>
       </c>
       <c r="B13" t="s">
+        <v>119</v>
+      </c>
+      <c r="C13" t="s">
+        <v>65</v>
+      </c>
+      <c r="D13" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="C13" t="s">
-        <v>66</v>
-      </c>
-      <c r="D13" s="3" t="s">
+      <c r="E13" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="E13" s="3" t="s">
+      <c r="F13" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="F13" s="3" t="s">
+      <c r="G13" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="G13" s="3" t="s">
+      <c r="H13" t="s">
         <v>124</v>
       </c>
-      <c r="H13" t="s">
+      <c r="I13" t="s">
         <v>125</v>
-      </c>
-      <c r="I13" t="s">
-        <v>126</v>
       </c>
       <c r="J13" s="9">
         <v>0</v>
@@ -5256,28 +5274,28 @@
         <v>91</v>
       </c>
       <c r="B14" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C14" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D14" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="E14" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="E14" s="3" t="s">
+      <c r="F14" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="F14" s="3" t="s">
+      <c r="G14" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="G14" s="3" t="s">
+      <c r="H14" t="s">
         <v>131</v>
       </c>
-      <c r="H14" t="s">
-        <v>132</v>
-      </c>
       <c r="I14" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="J14" s="9">
         <v>0.58333333333333337</v>
@@ -5318,28 +5336,28 @@
         <v>97</v>
       </c>
       <c r="B15" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C15" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D15" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E15" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="E15" s="3" t="s">
+      <c r="F15" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="F15" s="3" t="s">
+      <c r="G15" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="G15" s="3" t="s">
+      <c r="H15" t="s">
         <v>140</v>
       </c>
-      <c r="H15" t="s">
-        <v>141</v>
-      </c>
       <c r="I15" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="J15" s="9">
         <v>0.375</v>
@@ -5380,28 +5398,28 @@
         <v>110</v>
       </c>
       <c r="B16" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C16" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D16" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="E16" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="F16" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="F16" s="3" t="s">
+      <c r="G16" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="G16" s="3" t="s">
+      <c r="H16" t="s">
         <v>149</v>
       </c>
-      <c r="H16" t="s">
+      <c r="I16" t="s">
         <v>150</v>
-      </c>
-      <c r="I16" t="s">
-        <v>151</v>
       </c>
       <c r="J16" s="9">
         <v>0.55555555555555558</v>

</xml_diff>

<commit_message>
Results: neuer Zwischenstand (Hybrid + Sparse)
</commit_message>
<xml_diff>
--- a/src/evaluation/data/Backup/qwen25_7b_validation/comparison.xlsx
+++ b/src/evaluation/data/Backup/qwen25_7b_validation/comparison.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Uni-Köln\Masterarbeit\Software\uzk-masterarbeit\src\evaluation\data\Backup\qwen25_7b_validation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8EA6D8B-0322-4C8E-94FE-24C227AEE2DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54180B14-CA9B-4DCF-9F48-5482C81AA2C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>